<commit_message>
P6: declarar el alcance de la trazabilidad de RNF y RD
- matriz_e2e.xlsx: nota de alcance en A4 (42 RF + 18 RF-IA/RNF-IA
  trazados extremo a extremo; 19 RNF y 10 RD verificados por otra via)
- readme.md: seccion Alcance de las 73 filas
- AnexoA_auditoria_calidad.xlsx, hoja Valoracion, celda E8: acotado
  el criterio de M4 al alcance real medido (pendiente desde el cierre de P5)
- checksums.sha256 regenerado (191/191)
</commit_message>
<xml_diff>
--- a/AHMRV/04_Trazabilidad/matriz_e2e.xlsx
+++ b/AHMRV/04_Trazabilidad/matriz_e2e.xlsx
@@ -678,7 +678,13 @@
       </c>
       <c r="B3" s="31" t="n"/>
     </row>
-    <row r="4" ht="15" customHeight="1" s="32"/>
+    <row r="4" ht="15" customHeight="1" s="32">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ALCANCE. Esta matriz traza extremo a extremo los 42 RF y los 18 requisitos de IA (RF-IA/RNF-IA), 60 de 60. Los 19 RNF y los 10 RD del catálogo se verifican por otra vía (criterios de aceptación y revisión directa contra el ERS, no fila a fila en esta matriz); de ellos, 6 RNF y 2 RD sí tienen fila aquí porque además intervienen en una cadena funcional. Este alcance fue una decisión de auditoría de PE5, no un vacío de trazabilidad.</t>
+        </is>
+      </c>
+    </row>
     <row r="5" ht="15" customHeight="1" s="32"/>
     <row r="8" ht="23.25" customHeight="1" s="32">
       <c r="A8" s="36" t="inlineStr">

</xml_diff>